<commit_message>
v8.3: to-do leftovers; legacy bug L134 fixed in the prototype
TODO tidy (CPAT-team items merged, coded/TODO names); register spreadsheet
built from the register itself (identical table); excel_lint.check() after
every save of every Excel writer; leads closed (Manual inputs J178:J179 are
read; NOx forcing explained by the fixed L22/L23/L58/L59); new legacy bug
L134 (price-increase unit labels) fixed in ScenarioDefinition. Release v8.3:
quick check 0 change vs v8.2, paste test PASS; documents, tracker and deck
regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NEaWSMCoGDPkcQwasoKLW3
</commit_message>
<xml_diff>
--- a/excel_ai/legacy/workbooks/Tracking issues.xlsx
+++ b/excel_ai/legacy/workbooks/Tracking issues.xlsx
@@ -18,7 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPAT_dev" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BUGS'!$A$3:$T$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BUGS'!$A$3:$T$166</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ISSUES-OTHER'!$A$3:$T$150</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -1098,7 +1098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T165"/>
+  <dimension ref="A1:T166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1320,7 +1320,7 @@
       <c r="R4" s="58" t="inlineStr"/>
       <c r="S4" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T4" s="58" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="S5" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T5" s="58" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="S6" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T6" s="58" t="inlineStr">
@@ -1598,7 +1598,7 @@
       <c r="R7" s="58" t="inlineStr"/>
       <c r="S7" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T7" s="58" t="inlineStr">
@@ -1688,7 +1688,7 @@
       <c r="R8" s="58" t="inlineStr"/>
       <c r="S8" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T8" s="58" t="inlineStr">
@@ -1778,7 +1778,7 @@
       <c r="R9" s="58" t="inlineStr"/>
       <c r="S9" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T9" s="58" t="inlineStr">
@@ -1872,7 +1872,7 @@
       </c>
       <c r="S10" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T10" s="58" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="S11" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T11" s="58" t="inlineStr">
@@ -2056,7 +2056,7 @@
       <c r="R12" s="58" t="inlineStr"/>
       <c r="S12" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T12" s="58" t="inlineStr">
@@ -2146,7 +2146,7 @@
       <c r="R13" s="58" t="inlineStr"/>
       <c r="S13" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T13" s="58" t="inlineStr">
@@ -2240,7 +2240,7 @@
       <c r="R14" s="58" t="inlineStr"/>
       <c r="S14" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T14" s="58" t="inlineStr">
@@ -2330,7 +2330,7 @@
       <c r="R15" s="58" t="inlineStr"/>
       <c r="S15" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T15" s="58" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="S16" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T16" s="58" t="inlineStr">
@@ -2522,7 +2522,7 @@
       <c r="R17" s="58" t="inlineStr"/>
       <c r="S17" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T17" s="58" t="inlineStr">
@@ -2616,7 +2616,7 @@
       <c r="R18" s="58" t="inlineStr"/>
       <c r="S18" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T18" s="58" t="inlineStr">
@@ -2714,7 +2714,7 @@
       <c r="R19" s="58" t="inlineStr"/>
       <c r="S19" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T19" s="58" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="S20" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T20" s="58" t="inlineStr">
@@ -2906,7 +2906,7 @@
       <c r="R21" s="58" t="inlineStr"/>
       <c r="S21" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T21" s="58" t="inlineStr">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="S22" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T22" s="58" t="inlineStr">
@@ -3098,7 +3098,7 @@
       <c r="R23" s="58" t="inlineStr"/>
       <c r="S23" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T23" s="58" t="inlineStr">
@@ -3192,7 +3192,7 @@
       <c r="R24" s="58" t="inlineStr"/>
       <c r="S24" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T24" s="58" t="inlineStr">
@@ -3286,7 +3286,7 @@
       <c r="R25" s="58" t="inlineStr"/>
       <c r="S25" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T25" s="58" t="inlineStr">
@@ -3380,7 +3380,7 @@
       <c r="R26" s="58" t="inlineStr"/>
       <c r="S26" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T26" s="58" t="inlineStr">
@@ -3474,7 +3474,7 @@
       <c r="R27" s="58" t="inlineStr"/>
       <c r="S27" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T27" s="58" t="inlineStr">
@@ -3568,7 +3568,7 @@
       <c r="R28" s="58" t="inlineStr"/>
       <c r="S28" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T28" s="58" t="inlineStr">
@@ -3662,7 +3662,7 @@
       <c r="R29" s="58" t="inlineStr"/>
       <c r="S29" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T29" s="58" t="inlineStr">
@@ -3756,7 +3756,7 @@
       <c r="R30" s="58" t="inlineStr"/>
       <c r="S30" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T30" s="58" t="inlineStr">
@@ -3850,7 +3850,7 @@
       <c r="R31" s="58" t="inlineStr"/>
       <c r="S31" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T31" s="58" t="inlineStr">
@@ -3944,7 +3944,7 @@
       <c r="R32" s="58" t="inlineStr"/>
       <c r="S32" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T32" s="58" t="inlineStr">
@@ -4038,7 +4038,7 @@
       <c r="R33" s="58" t="inlineStr"/>
       <c r="S33" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T33" s="58" t="inlineStr">
@@ -4132,7 +4132,7 @@
       <c r="R34" s="58" t="inlineStr"/>
       <c r="S34" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T34" s="58" t="inlineStr">
@@ -4226,7 +4226,7 @@
       <c r="R35" s="58" t="inlineStr"/>
       <c r="S35" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T35" s="58" t="inlineStr">
@@ -4320,7 +4320,7 @@
       <c r="R36" s="58" t="inlineStr"/>
       <c r="S36" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T36" s="58" t="inlineStr">
@@ -4414,7 +4414,7 @@
       <c r="R37" s="58" t="inlineStr"/>
       <c r="S37" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T37" s="58" t="inlineStr">
@@ -4508,7 +4508,7 @@
       <c r="R38" s="58" t="inlineStr"/>
       <c r="S38" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T38" s="58" t="inlineStr">
@@ -4602,7 +4602,7 @@
       <c r="R39" s="58" t="inlineStr"/>
       <c r="S39" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T39" s="58" t="inlineStr">
@@ -4696,7 +4696,7 @@
       <c r="R40" s="58" t="inlineStr"/>
       <c r="S40" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T40" s="58" t="inlineStr">
@@ -4790,7 +4790,7 @@
       <c r="R41" s="58" t="inlineStr"/>
       <c r="S41" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T41" s="58" t="inlineStr">
@@ -4884,7 +4884,7 @@
       <c r="R42" s="58" t="inlineStr"/>
       <c r="S42" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T42" s="58" t="inlineStr">
@@ -4978,7 +4978,7 @@
       <c r="R43" s="58" t="inlineStr"/>
       <c r="S43" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T43" s="58" t="inlineStr">
@@ -5076,7 +5076,7 @@
       </c>
       <c r="S44" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T44" s="58" t="inlineStr">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="S45" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T45" s="58" t="inlineStr">
@@ -5260,7 +5260,7 @@
       <c r="R46" s="58" t="inlineStr"/>
       <c r="S46" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T46" s="58" t="inlineStr">
@@ -5358,7 +5358,7 @@
       <c r="R47" s="58" t="inlineStr"/>
       <c r="S47" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T47" s="58" t="inlineStr">
@@ -5448,7 +5448,7 @@
       <c r="R48" s="58" t="inlineStr"/>
       <c r="S48" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T48" s="58" t="inlineStr">
@@ -5538,7 +5538,7 @@
       <c r="R49" s="58" t="inlineStr"/>
       <c r="S49" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T49" s="58" t="inlineStr">
@@ -5636,7 +5636,7 @@
       </c>
       <c r="S50" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T50" s="58" t="inlineStr">
@@ -5730,7 +5730,7 @@
       <c r="R51" s="58" t="inlineStr"/>
       <c r="S51" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T51" s="58" t="inlineStr">
@@ -5824,7 +5824,7 @@
       <c r="R52" s="58" t="inlineStr"/>
       <c r="S52" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T52" s="58" t="inlineStr">
@@ -5918,7 +5918,7 @@
       <c r="R53" s="58" t="inlineStr"/>
       <c r="S53" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T53" s="58" t="inlineStr">
@@ -6012,7 +6012,7 @@
       <c r="R54" s="58" t="inlineStr"/>
       <c r="S54" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T54" s="58" t="inlineStr">
@@ -6106,7 +6106,7 @@
       <c r="R55" s="58" t="inlineStr"/>
       <c r="S55" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T55" s="58" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="S56" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T56" s="58" t="inlineStr">
@@ -6298,7 +6298,7 @@
       <c r="R57" s="58" t="inlineStr"/>
       <c r="S57" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T57" s="58" t="inlineStr">
@@ -6396,7 +6396,7 @@
       <c r="R58" s="58" t="inlineStr"/>
       <c r="S58" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T58" s="58" t="inlineStr">
@@ -6494,7 +6494,7 @@
       <c r="R59" s="58" t="inlineStr"/>
       <c r="S59" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T59" s="58" t="inlineStr">
@@ -6588,7 +6588,7 @@
       <c r="R60" s="58" t="inlineStr"/>
       <c r="S60" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T60" s="58" t="inlineStr">
@@ -6682,7 +6682,7 @@
       <c r="R61" s="58" t="inlineStr"/>
       <c r="S61" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T61" s="58" t="inlineStr">
@@ -6776,7 +6776,7 @@
       <c r="R62" s="58" t="inlineStr"/>
       <c r="S62" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T62" s="58" t="inlineStr">
@@ -6870,7 +6870,7 @@
       <c r="R63" s="58" t="inlineStr"/>
       <c r="S63" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T63" s="58" t="inlineStr">
@@ -6968,7 +6968,7 @@
       <c r="R64" s="58" t="inlineStr"/>
       <c r="S64" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T64" s="58" t="inlineStr">
@@ -7066,7 +7066,7 @@
       <c r="R65" s="58" t="inlineStr"/>
       <c r="S65" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T65" s="58" t="inlineStr">
@@ -7160,7 +7160,7 @@
       <c r="R66" s="58" t="inlineStr"/>
       <c r="S66" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T66" s="58" t="inlineStr">
@@ -7254,7 +7254,7 @@
       <c r="R67" s="58" t="inlineStr"/>
       <c r="S67" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T67" s="58" t="inlineStr">
@@ -7348,7 +7348,7 @@
       <c r="R68" s="58" t="inlineStr"/>
       <c r="S68" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T68" s="58" t="inlineStr">
@@ -7442,7 +7442,7 @@
       <c r="R69" s="58" t="inlineStr"/>
       <c r="S69" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T69" s="58" t="inlineStr">
@@ -7536,7 +7536,7 @@
       <c r="R70" s="58" t="inlineStr"/>
       <c r="S70" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T70" s="58" t="inlineStr">
@@ -7626,7 +7626,7 @@
       <c r="R71" s="58" t="inlineStr"/>
       <c r="S71" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T71" s="58" t="inlineStr">
@@ -7720,7 +7720,7 @@
       <c r="R72" s="58" t="inlineStr"/>
       <c r="S72" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T72" s="58" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="S73" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T73" s="58" t="inlineStr">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="S74" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T74" s="58" t="inlineStr">
@@ -7998,7 +7998,7 @@
       <c r="R75" s="58" t="inlineStr"/>
       <c r="S75" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T75" s="58" t="inlineStr">
@@ -8092,7 +8092,7 @@
       <c r="R76" s="58" t="inlineStr"/>
       <c r="S76" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T76" s="58" t="inlineStr">
@@ -8186,7 +8186,7 @@
       <c r="R77" s="58" t="inlineStr"/>
       <c r="S77" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T77" s="58" t="inlineStr">
@@ -8284,7 +8284,7 @@
       </c>
       <c r="S78" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T78" s="58" t="inlineStr">
@@ -8378,7 +8378,7 @@
       <c r="R79" s="58" t="inlineStr"/>
       <c r="S79" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T79" s="58" t="inlineStr">
@@ -8472,7 +8472,7 @@
       <c r="R80" s="58" t="inlineStr"/>
       <c r="S80" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T80" s="58" t="inlineStr">
@@ -8562,7 +8562,7 @@
       <c r="R81" s="58" t="inlineStr"/>
       <c r="S81" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T81" s="58" t="inlineStr">
@@ -8656,7 +8656,7 @@
       <c r="R82" s="58" t="inlineStr"/>
       <c r="S82" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T82" s="58" t="inlineStr">
@@ -8750,7 +8750,7 @@
       <c r="R83" s="58" t="inlineStr"/>
       <c r="S83" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T83" s="58" t="inlineStr">
@@ -8848,7 +8848,7 @@
       <c r="R84" s="58" t="inlineStr"/>
       <c r="S84" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T84" s="58" t="inlineStr">
@@ -8942,7 +8942,7 @@
       <c r="R85" s="58" t="inlineStr"/>
       <c r="S85" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T85" s="58" t="inlineStr">
@@ -9032,7 +9032,7 @@
       <c r="R86" s="58" t="inlineStr"/>
       <c r="S86" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T86" s="58" t="inlineStr">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="S87" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T87" s="58" t="inlineStr">
@@ -9224,7 +9224,7 @@
       <c r="R88" s="58" t="inlineStr"/>
       <c r="S88" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T88" s="58" t="inlineStr">
@@ -9318,7 +9318,7 @@
       <c r="R89" s="58" t="inlineStr"/>
       <c r="S89" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T89" s="58" t="inlineStr">
@@ -9408,7 +9408,7 @@
       <c r="R90" s="58" t="inlineStr"/>
       <c r="S90" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T90" s="58" t="inlineStr">
@@ -9510,7 +9510,7 @@
       </c>
       <c r="S91" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T91" s="58" t="inlineStr">
@@ -9608,7 +9608,7 @@
       </c>
       <c r="S92" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T92" s="58" t="inlineStr">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="S93" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T93" s="58" t="inlineStr">
@@ -9796,7 +9796,7 @@
       </c>
       <c r="S94" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T94" s="58" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="S95" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T95" s="58" t="inlineStr">
@@ -9984,7 +9984,7 @@
       </c>
       <c r="S96" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T96" s="58" t="inlineStr">
@@ -10078,7 +10078,7 @@
       </c>
       <c r="S97" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T97" s="58" t="inlineStr">
@@ -10172,7 +10172,7 @@
       </c>
       <c r="S98" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T98" s="58" t="inlineStr">
@@ -10266,7 +10266,7 @@
       </c>
       <c r="S99" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T99" s="58" t="inlineStr">
@@ -10360,7 +10360,7 @@
       </c>
       <c r="S100" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T100" s="58" t="inlineStr">
@@ -10454,7 +10454,7 @@
       </c>
       <c r="S101" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T101" s="58" t="inlineStr">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="S102" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T102" s="58" t="inlineStr">
@@ -10646,7 +10646,7 @@
       <c r="R103" s="58" t="inlineStr"/>
       <c r="S103" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T103" s="58" t="inlineStr">
@@ -10740,7 +10740,7 @@
       <c r="R104" s="58" t="inlineStr"/>
       <c r="S104" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T104" s="58" t="inlineStr">
@@ -10834,7 +10834,7 @@
       <c r="R105" s="58" t="inlineStr"/>
       <c r="S105" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T105" s="58" t="inlineStr">
@@ -10924,7 +10924,7 @@
       <c r="R106" s="58" t="inlineStr"/>
       <c r="S106" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T106" s="58" t="inlineStr">
@@ -11014,7 +11014,7 @@
       <c r="R107" s="58" t="inlineStr"/>
       <c r="S107" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T107" s="58" t="inlineStr">
@@ -11104,7 +11104,7 @@
       <c r="R108" s="58" t="inlineStr"/>
       <c r="S108" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T108" s="58" t="inlineStr">
@@ -11194,7 +11194,7 @@
       <c r="R109" s="58" t="inlineStr"/>
       <c r="S109" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T109" s="58" t="inlineStr">
@@ -11284,7 +11284,7 @@
       <c r="R110" s="58" t="inlineStr"/>
       <c r="S110" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T110" s="58" t="inlineStr">
@@ -11374,7 +11374,7 @@
       <c r="R111" s="58" t="inlineStr"/>
       <c r="S111" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T111" s="58" t="inlineStr">
@@ -11468,7 +11468,7 @@
       <c r="R112" s="58" t="inlineStr"/>
       <c r="S112" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T112" s="58" t="inlineStr">
@@ -11562,7 +11562,7 @@
       <c r="R113" s="58" t="inlineStr"/>
       <c r="S113" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T113" s="58" t="inlineStr">
@@ -11652,7 +11652,7 @@
       <c r="R114" s="58" t="inlineStr"/>
       <c r="S114" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T114" s="58" t="inlineStr">
@@ -11742,7 +11742,7 @@
       <c r="R115" s="58" t="inlineStr"/>
       <c r="S115" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T115" s="58" t="inlineStr">
@@ -11832,7 +11832,7 @@
       <c r="R116" s="58" t="inlineStr"/>
       <c r="S116" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T116" s="58" t="inlineStr">
@@ -11926,7 +11926,7 @@
       <c r="R117" s="58" t="inlineStr"/>
       <c r="S117" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T117" s="58" t="inlineStr">
@@ -12020,7 +12020,7 @@
       <c r="R118" s="58" t="inlineStr"/>
       <c r="S118" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T118" s="58" t="inlineStr">
@@ -12118,7 +12118,7 @@
       <c r="R119" s="58" t="inlineStr"/>
       <c r="S119" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T119" s="58" t="inlineStr">
@@ -12212,7 +12212,7 @@
       <c r="R120" s="58" t="inlineStr"/>
       <c r="S120" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T120" s="58" t="inlineStr">
@@ -12306,7 +12306,7 @@
       <c r="R121" s="58" t="inlineStr"/>
       <c r="S121" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T121" s="58" t="inlineStr">
@@ -12404,7 +12404,7 @@
       <c r="R122" s="58" t="inlineStr"/>
       <c r="S122" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T122" s="58" t="inlineStr">
@@ -12498,7 +12498,7 @@
       <c r="R123" s="58" t="inlineStr"/>
       <c r="S123" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T123" s="58" t="inlineStr">
@@ -12592,7 +12592,7 @@
       <c r="R124" s="58" t="inlineStr"/>
       <c r="S124" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T124" s="58" t="inlineStr">
@@ -12686,7 +12686,7 @@
       <c r="R125" s="58" t="inlineStr"/>
       <c r="S125" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T125" s="58" t="inlineStr">
@@ -12776,7 +12776,7 @@
       <c r="R126" s="58" t="inlineStr"/>
       <c r="S126" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T126" s="58" t="inlineStr">
@@ -12866,7 +12866,7 @@
       <c r="R127" s="58" t="inlineStr"/>
       <c r="S127" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T127" s="58" t="inlineStr">
@@ -12960,7 +12960,7 @@
       <c r="R128" s="58" t="inlineStr"/>
       <c r="S128" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T128" s="58" t="inlineStr">
@@ -13054,7 +13054,7 @@
       <c r="R129" s="58" t="inlineStr"/>
       <c r="S129" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T129" s="58" t="inlineStr">
@@ -13148,7 +13148,7 @@
       <c r="R130" s="58" t="inlineStr"/>
       <c r="S130" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T130" s="58" t="inlineStr">
@@ -13242,7 +13242,7 @@
       <c r="R131" s="58" t="inlineStr"/>
       <c r="S131" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T131" s="58" t="inlineStr">
@@ -13336,7 +13336,7 @@
       <c r="R132" s="58" t="inlineStr"/>
       <c r="S132" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T132" s="58" t="inlineStr">
@@ -13430,7 +13430,7 @@
       <c r="R133" s="58" t="inlineStr"/>
       <c r="S133" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T133" s="58" t="inlineStr">
@@ -13520,7 +13520,7 @@
       <c r="R134" s="58" t="inlineStr"/>
       <c r="S134" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T134" s="58" t="inlineStr">
@@ -13610,7 +13610,7 @@
       <c r="R135" s="58" t="inlineStr"/>
       <c r="S135" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T135" s="58" t="inlineStr">
@@ -13700,7 +13700,7 @@
       <c r="R136" s="58" t="inlineStr"/>
       <c r="S136" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T136" s="58" t="inlineStr">
@@ -13790,7 +13790,7 @@
       <c r="R137" s="58" t="inlineStr"/>
       <c r="S137" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T137" s="58" t="inlineStr">
@@ -13880,7 +13880,7 @@
       <c r="R138" s="58" t="inlineStr"/>
       <c r="S138" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T138" s="58" t="inlineStr">
@@ -13970,7 +13970,7 @@
       <c r="R139" s="58" t="inlineStr"/>
       <c r="S139" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T139" s="58" t="inlineStr">
@@ -14056,7 +14056,7 @@
       <c r="R140" s="58" t="inlineStr"/>
       <c r="S140" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T140" s="58" t="inlineStr">
@@ -14146,7 +14146,7 @@
       <c r="R141" s="58" t="inlineStr"/>
       <c r="S141" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T141" s="58" t="inlineStr">
@@ -14236,7 +14236,7 @@
       <c r="R142" s="58" t="inlineStr"/>
       <c r="S142" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T142" s="58" t="inlineStr">
@@ -14326,7 +14326,7 @@
       <c r="R143" s="58" t="inlineStr"/>
       <c r="S143" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T143" s="58" t="inlineStr">
@@ -14416,7 +14416,7 @@
       <c r="R144" s="58" t="inlineStr"/>
       <c r="S144" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T144" s="58" t="inlineStr">
@@ -14506,7 +14506,7 @@
       <c r="R145" s="58" t="inlineStr"/>
       <c r="S145" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T145" s="58" t="inlineStr">
@@ -14596,7 +14596,7 @@
       <c r="R146" s="58" t="inlineStr"/>
       <c r="S146" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T146" s="58" t="inlineStr">
@@ -14686,7 +14686,7 @@
       <c r="R147" s="58" t="inlineStr"/>
       <c r="S147" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T147" s="58" t="inlineStr">
@@ -14776,7 +14776,7 @@
       <c r="R148" s="58" t="inlineStr"/>
       <c r="S148" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T148" s="58" t="inlineStr">
@@ -14866,7 +14866,7 @@
       <c r="R149" s="58" t="inlineStr"/>
       <c r="S149" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T149" s="58" t="inlineStr">
@@ -14956,7 +14956,7 @@
       <c r="R150" s="58" t="inlineStr"/>
       <c r="S150" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T150" s="58" t="inlineStr">
@@ -15046,7 +15046,7 @@
       <c r="R151" s="58" t="inlineStr"/>
       <c r="S151" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T151" s="58" t="inlineStr">
@@ -15132,7 +15132,7 @@
       <c r="R152" s="58" t="inlineStr"/>
       <c r="S152" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T152" s="58" t="inlineStr">
@@ -15222,7 +15222,7 @@
       <c r="R153" s="58" t="inlineStr"/>
       <c r="S153" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T153" s="58" t="inlineStr">
@@ -15312,7 +15312,7 @@
       <c r="R154" s="58" t="inlineStr"/>
       <c r="S154" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T154" s="58" t="inlineStr">
@@ -15398,7 +15398,7 @@
       <c r="R155" s="58" t="inlineStr"/>
       <c r="S155" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T155" s="58" t="inlineStr">
@@ -15496,7 +15496,7 @@
       <c r="R156" s="58" t="inlineStr"/>
       <c r="S156" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T156" s="58" t="inlineStr">
@@ -15594,7 +15594,7 @@
       <c r="R157" s="58" t="inlineStr"/>
       <c r="S157" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T157" s="58" t="inlineStr">
@@ -15688,7 +15688,7 @@
       <c r="R158" s="58" t="inlineStr"/>
       <c r="S158" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T158" s="58" t="inlineStr">
@@ -15782,7 +15782,7 @@
       <c r="R159" s="58" t="inlineStr"/>
       <c r="S159" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T159" s="58" t="inlineStr">
@@ -15876,7 +15876,7 @@
       <c r="R160" s="58" t="inlineStr"/>
       <c r="S160" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T160" s="58" t="inlineStr">
@@ -15962,7 +15962,7 @@
       <c r="R161" s="58" t="inlineStr"/>
       <c r="S161" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T161" s="58" t="inlineStr">
@@ -16048,7 +16048,7 @@
       <c r="R162" s="58" t="inlineStr"/>
       <c r="S162" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T162" s="58" t="inlineStr">
@@ -16138,7 +16138,7 @@
       <c r="R163" s="58" t="inlineStr"/>
       <c r="S163" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T163" s="58" t="inlineStr">
@@ -16228,7 +16228,7 @@
       <c r="R164" s="58" t="inlineStr"/>
       <c r="S164" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T164" s="58" t="inlineStr">
@@ -16318,7 +16318,7 @@
       <c r="R165" s="58" t="inlineStr"/>
       <c r="S165" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T165" s="58" t="inlineStr">
@@ -16327,15 +16327,105 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" s="58" t="inlineStr">
+        <is>
+          <t>L134</t>
+        </is>
+      </c>
+      <c r="B166" s="58" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C166" s="58" t="inlineStr"/>
+      <c r="D166" s="58" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E166" s="58" t="inlineStr">
+        <is>
+          <t>Price-increase units: other oil products "$/bbn", default "$/liter" for other oil products and biomass</t>
+        </is>
+      </c>
+      <c r="F166" s="58" t="inlineStr">
+        <is>
+          <t>Legacy bug (mitigation)</t>
+        </is>
+      </c>
+      <c r="G166" s="58" t="inlineStr">
+        <is>
+          <t>Other mitigation</t>
+        </is>
+      </c>
+      <c r="H166" s="58" t="inlineStr">
+        <is>
+          <t>MTInputs rows 182-183 (columns E and G); Mitigation I177, I180</t>
+        </is>
+      </c>
+      <c r="I166" s="58" t="inlineStr">
+        <is>
+          <t>The unit labels of the price-increase inputs read "$/bbn" (for $/bbl) for other oil products, and the default column says "$/liter" for other oil products and biomass, whose prices are per barrel and per GJ. No formula reads the labels (Mitigation rows 168-180 use the amounts in G and H only), so no value changes; a user typing an increase per liter for these fuels gets a wrong price path. Found by the tracker leads (2026-10-23).</t>
+        </is>
+      </c>
+      <c r="J166" s="58" t="inlineStr">
+        <is>
+          <t>Label the price-increase units USD/bbl (other oil products) and USD/GJ (biomass) in columns E and G of MTInputs rows 182-183.</t>
+        </is>
+      </c>
+      <c r="K166" s="58" t="inlineStr">
+        <is>
+          <t>Labels only: no value changes; a user may type an increase in the wrong unit. prototype: Fixed (v8.3): the prototype's ScenarioDefinition rows 182-183 read $/bbl and $/GJ, defaults included.</t>
+        </is>
+      </c>
+      <c r="L166" s="58" t="inlineStr"/>
+      <c r="M166" s="58" t="inlineStr">
+        <is>
+          <t>Not reconciled yet</t>
+        </is>
+      </c>
+      <c r="N166" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O166" s="58" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="P166" s="58" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q166" s="58" t="inlineStr">
+        <is>
+          <t>8.3</t>
+        </is>
+      </c>
+      <c r="R166" s="58" t="inlineStr"/>
+      <c r="S166" s="58" t="inlineStr">
+        <is>
+          <t>v8.3</t>
+        </is>
+      </c>
+      <c r="T166" s="58" t="inlineStr">
+        <is>
+          <t>Legacy bug</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:T165">
+  <autoFilter ref="A3:T166">
     <filterColumn colId="1" hiddenButton="0" showButton="1">
       <customFilters>
         <customFilter val="Closed*" operator="notEqual"/>
       </customFilters>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A4:T165">
+  <conditionalFormatting sqref="A4:T166">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>LEFT($B4,6)="Closed"</formula>
     </cfRule>
@@ -16568,7 +16658,7 @@
       <c r="R4" s="58" t="inlineStr"/>
       <c r="S4" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T4" s="58" t="inlineStr">
@@ -16650,7 +16740,7 @@
       <c r="R5" s="58" t="inlineStr"/>
       <c r="S5" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T5" s="58" t="inlineStr">
@@ -16740,7 +16830,7 @@
       </c>
       <c r="S6" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T6" s="58" t="inlineStr">
@@ -16822,7 +16912,7 @@
       <c r="R7" s="58" t="inlineStr"/>
       <c r="S7" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T7" s="58" t="inlineStr">
@@ -16908,7 +16998,7 @@
       <c r="R8" s="58" t="inlineStr"/>
       <c r="S8" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T8" s="58" t="inlineStr">
@@ -16990,7 +17080,7 @@
       <c r="R9" s="58" t="inlineStr"/>
       <c r="S9" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T9" s="58" t="inlineStr">
@@ -17072,7 +17162,7 @@
       <c r="R10" s="58" t="inlineStr"/>
       <c r="S10" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T10" s="58" t="inlineStr">
@@ -17158,7 +17248,7 @@
       <c r="R11" s="58" t="inlineStr"/>
       <c r="S11" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T11" s="58" t="inlineStr">
@@ -17244,7 +17334,7 @@
       <c r="R12" s="58" t="inlineStr"/>
       <c r="S12" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T12" s="58" t="inlineStr">
@@ -17326,7 +17416,7 @@
       <c r="R13" s="58" t="inlineStr"/>
       <c r="S13" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T13" s="58" t="inlineStr">
@@ -17416,7 +17506,7 @@
       </c>
       <c r="S14" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T14" s="58" t="inlineStr">
@@ -17502,7 +17592,7 @@
       <c r="R15" s="58" t="inlineStr"/>
       <c r="S15" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T15" s="58" t="inlineStr">
@@ -17588,7 +17678,7 @@
       <c r="R16" s="58" t="inlineStr"/>
       <c r="S16" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T16" s="58" t="inlineStr">
@@ -17670,7 +17760,7 @@
       <c r="R17" s="58" t="inlineStr"/>
       <c r="S17" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T17" s="58" t="inlineStr">
@@ -17756,7 +17846,7 @@
       <c r="R18" s="58" t="inlineStr"/>
       <c r="S18" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T18" s="58" t="inlineStr">
@@ -17846,7 +17936,7 @@
       <c r="R19" s="58" t="inlineStr"/>
       <c r="S19" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T19" s="58" t="inlineStr">
@@ -17936,7 +18026,7 @@
       </c>
       <c r="S20" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T20" s="58" t="inlineStr">
@@ -18022,7 +18112,7 @@
       <c r="R21" s="58" t="inlineStr"/>
       <c r="S21" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T21" s="58" t="inlineStr">
@@ -18108,7 +18198,7 @@
       </c>
       <c r="S22" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T22" s="58" t="inlineStr">
@@ -18194,7 +18284,7 @@
       <c r="R23" s="58" t="inlineStr"/>
       <c r="S23" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T23" s="58" t="inlineStr">
@@ -18280,7 +18370,7 @@
       <c r="R24" s="58" t="inlineStr"/>
       <c r="S24" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T24" s="58" t="inlineStr">
@@ -18366,7 +18456,7 @@
       <c r="R25" s="58" t="inlineStr"/>
       <c r="S25" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T25" s="58" t="inlineStr">
@@ -18452,7 +18542,7 @@
       <c r="R26" s="58" t="inlineStr"/>
       <c r="S26" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T26" s="58" t="inlineStr">
@@ -18530,7 +18620,7 @@
       <c r="R27" s="58" t="inlineStr"/>
       <c r="S27" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T27" s="58" t="inlineStr">
@@ -18612,7 +18702,7 @@
       </c>
       <c r="S28" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T28" s="58" t="inlineStr">
@@ -18694,7 +18784,7 @@
       <c r="R29" s="58" t="inlineStr"/>
       <c r="S29" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T29" s="58" t="inlineStr">
@@ -18772,7 +18862,7 @@
       <c r="R30" s="58" t="inlineStr"/>
       <c r="S30" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T30" s="58" t="inlineStr">
@@ -18854,7 +18944,7 @@
       <c r="R31" s="58" t="inlineStr"/>
       <c r="S31" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T31" s="58" t="inlineStr">
@@ -18936,7 +19026,7 @@
       <c r="R32" s="58" t="inlineStr"/>
       <c r="S32" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T32" s="58" t="inlineStr">
@@ -19022,7 +19112,7 @@
       <c r="R33" s="58" t="inlineStr"/>
       <c r="S33" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T33" s="58" t="inlineStr">
@@ -19104,7 +19194,7 @@
       <c r="R34" s="58" t="inlineStr"/>
       <c r="S34" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T34" s="58" t="inlineStr">
@@ -19190,7 +19280,7 @@
       </c>
       <c r="S35" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T35" s="58" t="inlineStr">
@@ -19268,7 +19358,7 @@
       <c r="R36" s="58" t="inlineStr"/>
       <c r="S36" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T36" s="58" t="inlineStr">
@@ -19346,7 +19436,7 @@
       <c r="R37" s="58" t="inlineStr"/>
       <c r="S37" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T37" s="58" t="inlineStr">
@@ -19424,7 +19514,7 @@
       <c r="R38" s="58" t="inlineStr"/>
       <c r="S38" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T38" s="58" t="inlineStr">
@@ -19506,7 +19596,7 @@
       </c>
       <c r="S39" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T39" s="58" t="inlineStr">
@@ -19584,7 +19674,7 @@
       <c r="R40" s="58" t="inlineStr"/>
       <c r="S40" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T40" s="58" t="inlineStr">
@@ -19666,7 +19756,7 @@
       <c r="R41" s="58" t="inlineStr"/>
       <c r="S41" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T41" s="58" t="inlineStr">
@@ -19748,7 +19838,7 @@
       <c r="R42" s="58" t="inlineStr"/>
       <c r="S42" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T42" s="58" t="inlineStr">
@@ -19830,7 +19920,7 @@
       <c r="R43" s="58" t="inlineStr"/>
       <c r="S43" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T43" s="58" t="inlineStr">
@@ -19912,7 +20002,7 @@
       <c r="R44" s="58" t="inlineStr"/>
       <c r="S44" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T44" s="58" t="inlineStr">
@@ -19998,7 +20088,7 @@
       <c r="R45" s="58" t="inlineStr"/>
       <c r="S45" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T45" s="58" t="inlineStr">
@@ -20080,7 +20170,7 @@
       <c r="R46" s="58" t="inlineStr"/>
       <c r="S46" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T46" s="58" t="inlineStr">
@@ -20166,7 +20256,7 @@
       </c>
       <c r="S47" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T47" s="58" t="inlineStr">
@@ -20248,7 +20338,7 @@
       <c r="R48" s="58" t="inlineStr"/>
       <c r="S48" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T48" s="58" t="inlineStr">
@@ -20330,7 +20420,7 @@
       <c r="R49" s="58" t="inlineStr"/>
       <c r="S49" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T49" s="58" t="inlineStr">
@@ -20408,7 +20498,7 @@
       <c r="R50" s="58" t="inlineStr"/>
       <c r="S50" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T50" s="58" t="inlineStr">
@@ -20494,7 +20584,7 @@
       <c r="R51" s="58" t="inlineStr"/>
       <c r="S51" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T51" s="58" t="inlineStr">
@@ -20580,7 +20670,7 @@
       <c r="R52" s="58" t="inlineStr"/>
       <c r="S52" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T52" s="58" t="inlineStr">
@@ -20666,7 +20756,7 @@
       <c r="R53" s="58" t="inlineStr"/>
       <c r="S53" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T53" s="58" t="inlineStr">
@@ -20748,7 +20838,7 @@
       <c r="R54" s="58" t="inlineStr"/>
       <c r="S54" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T54" s="58" t="inlineStr">
@@ -20834,7 +20924,7 @@
       </c>
       <c r="S55" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T55" s="58" t="inlineStr">
@@ -20916,7 +21006,7 @@
       <c r="R56" s="58" t="inlineStr"/>
       <c r="S56" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T56" s="58" t="inlineStr">
@@ -21002,7 +21092,7 @@
       <c r="R57" s="58" t="inlineStr"/>
       <c r="S57" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T57" s="58" t="inlineStr">
@@ -21084,7 +21174,7 @@
       <c r="R58" s="58" t="inlineStr"/>
       <c r="S58" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T58" s="58" t="inlineStr">
@@ -21162,7 +21252,7 @@
       <c r="R59" s="58" t="inlineStr"/>
       <c r="S59" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T59" s="58" t="inlineStr">
@@ -21244,7 +21334,7 @@
       <c r="R60" s="58" t="inlineStr"/>
       <c r="S60" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T60" s="58" t="inlineStr">
@@ -21326,7 +21416,7 @@
       <c r="R61" s="58" t="inlineStr"/>
       <c r="S61" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T61" s="58" t="inlineStr">
@@ -21408,7 +21498,7 @@
       <c r="R62" s="58" t="inlineStr"/>
       <c r="S62" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T62" s="58" t="inlineStr">
@@ -21490,7 +21580,7 @@
       <c r="R63" s="58" t="inlineStr"/>
       <c r="S63" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T63" s="58" t="inlineStr">
@@ -21576,7 +21666,7 @@
       <c r="R64" s="58" t="inlineStr"/>
       <c r="S64" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T64" s="58" t="inlineStr">
@@ -21654,7 +21744,7 @@
       <c r="R65" s="58" t="inlineStr"/>
       <c r="S65" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T65" s="58" t="inlineStr">
@@ -21736,7 +21826,7 @@
       </c>
       <c r="S66" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T66" s="58" t="inlineStr">
@@ -21814,7 +21904,7 @@
       <c r="R67" s="58" t="inlineStr"/>
       <c r="S67" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T67" s="58" t="inlineStr">
@@ -21892,7 +21982,7 @@
       <c r="R68" s="58" t="inlineStr"/>
       <c r="S68" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T68" s="58" t="inlineStr">
@@ -21974,7 +22064,7 @@
       <c r="R69" s="58" t="inlineStr"/>
       <c r="S69" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T69" s="58" t="inlineStr">
@@ -22052,7 +22142,7 @@
       <c r="R70" s="58" t="inlineStr"/>
       <c r="S70" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T70" s="58" t="inlineStr">
@@ -22130,7 +22220,7 @@
       <c r="R71" s="58" t="inlineStr"/>
       <c r="S71" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T71" s="58" t="inlineStr">
@@ -22212,7 +22302,7 @@
       <c r="R72" s="58" t="inlineStr"/>
       <c r="S72" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T72" s="58" t="inlineStr">
@@ -22290,7 +22380,7 @@
       <c r="R73" s="58" t="inlineStr"/>
       <c r="S73" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T73" s="58" t="inlineStr">
@@ -22372,7 +22462,7 @@
       <c r="R74" s="58" t="inlineStr"/>
       <c r="S74" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T74" s="58" t="inlineStr">
@@ -22454,7 +22544,7 @@
       <c r="R75" s="58" t="inlineStr"/>
       <c r="S75" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T75" s="58" t="inlineStr">
@@ -22532,7 +22622,7 @@
       <c r="R76" s="58" t="inlineStr"/>
       <c r="S76" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T76" s="58" t="inlineStr">
@@ -22610,7 +22700,7 @@
       <c r="R77" s="58" t="inlineStr"/>
       <c r="S77" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T77" s="58" t="inlineStr">
@@ -22688,7 +22778,7 @@
       <c r="R78" s="58" t="inlineStr"/>
       <c r="S78" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T78" s="58" t="inlineStr">
@@ -22770,7 +22860,7 @@
       </c>
       <c r="S79" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T79" s="58" t="inlineStr">
@@ -22852,7 +22942,7 @@
       <c r="R80" s="58" t="inlineStr"/>
       <c r="S80" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T80" s="58" t="inlineStr">
@@ -22934,7 +23024,7 @@
       <c r="R81" s="58" t="inlineStr"/>
       <c r="S81" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T81" s="58" t="inlineStr">
@@ -23012,7 +23102,7 @@
       <c r="R82" s="58" t="inlineStr"/>
       <c r="S82" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T82" s="58" t="inlineStr">
@@ -23102,7 +23192,7 @@
       <c r="R83" s="58" t="inlineStr"/>
       <c r="S83" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T83" s="58" t="inlineStr">
@@ -23188,7 +23278,7 @@
       <c r="R84" s="58" t="inlineStr"/>
       <c r="S84" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T84" s="58" t="inlineStr">
@@ -23274,7 +23364,7 @@
       <c r="R85" s="58" t="inlineStr"/>
       <c r="S85" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T85" s="58" t="inlineStr">
@@ -23356,7 +23446,7 @@
       <c r="R86" s="58" t="inlineStr"/>
       <c r="S86" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T86" s="58" t="inlineStr">
@@ -23438,7 +23528,7 @@
       <c r="R87" s="58" t="inlineStr"/>
       <c r="S87" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T87" s="58" t="inlineStr">
@@ -23520,7 +23610,7 @@
       <c r="R88" s="58" t="inlineStr"/>
       <c r="S88" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T88" s="58" t="inlineStr">
@@ -23602,7 +23692,7 @@
       <c r="R89" s="58" t="inlineStr"/>
       <c r="S89" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T89" s="58" t="inlineStr">
@@ -23684,7 +23774,7 @@
       <c r="R90" s="58" t="inlineStr"/>
       <c r="S90" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T90" s="58" t="inlineStr">
@@ -23766,7 +23856,7 @@
       <c r="R91" s="58" t="inlineStr"/>
       <c r="S91" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T91" s="58" t="inlineStr">
@@ -23848,7 +23938,7 @@
       <c r="R92" s="58" t="inlineStr"/>
       <c r="S92" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T92" s="58" t="inlineStr">
@@ -23930,7 +24020,7 @@
       <c r="R93" s="58" t="inlineStr"/>
       <c r="S93" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T93" s="58" t="inlineStr">
@@ -24012,7 +24102,7 @@
       <c r="R94" s="58" t="inlineStr"/>
       <c r="S94" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T94" s="58" t="inlineStr">
@@ -24094,7 +24184,7 @@
       <c r="R95" s="58" t="inlineStr"/>
       <c r="S95" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T95" s="58" t="inlineStr">
@@ -24176,7 +24266,7 @@
       <c r="R96" s="58" t="inlineStr"/>
       <c r="S96" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T96" s="58" t="inlineStr">
@@ -24258,7 +24348,7 @@
       <c r="R97" s="58" t="inlineStr"/>
       <c r="S97" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T97" s="58" t="inlineStr">
@@ -24340,7 +24430,7 @@
       <c r="R98" s="58" t="inlineStr"/>
       <c r="S98" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T98" s="58" t="inlineStr">
@@ -24426,7 +24516,7 @@
       <c r="R99" s="58" t="inlineStr"/>
       <c r="S99" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T99" s="58" t="inlineStr">
@@ -24512,7 +24602,7 @@
       <c r="R100" s="58" t="inlineStr"/>
       <c r="S100" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T100" s="58" t="inlineStr">
@@ -24598,7 +24688,7 @@
       <c r="R101" s="58" t="inlineStr"/>
       <c r="S101" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T101" s="58" t="inlineStr">
@@ -24684,7 +24774,7 @@
       <c r="R102" s="58" t="inlineStr"/>
       <c r="S102" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T102" s="58" t="inlineStr">
@@ -24770,7 +24860,7 @@
       <c r="R103" s="58" t="inlineStr"/>
       <c r="S103" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T103" s="58" t="inlineStr">
@@ -24856,7 +24946,7 @@
       <c r="R104" s="58" t="inlineStr"/>
       <c r="S104" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T104" s="58" t="inlineStr">
@@ -24942,7 +25032,7 @@
       <c r="R105" s="58" t="inlineStr"/>
       <c r="S105" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T105" s="58" t="inlineStr">
@@ -25028,7 +25118,7 @@
       <c r="R106" s="58" t="inlineStr"/>
       <c r="S106" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T106" s="58" t="inlineStr">
@@ -25114,7 +25204,7 @@
       <c r="R107" s="58" t="inlineStr"/>
       <c r="S107" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T107" s="58" t="inlineStr">
@@ -25200,7 +25290,7 @@
       <c r="R108" s="58" t="inlineStr"/>
       <c r="S108" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T108" s="58" t="inlineStr">
@@ -25286,7 +25376,7 @@
       <c r="R109" s="58" t="inlineStr"/>
       <c r="S109" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T109" s="58" t="inlineStr">
@@ -25372,7 +25462,7 @@
       <c r="R110" s="58" t="inlineStr"/>
       <c r="S110" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T110" s="58" t="inlineStr">
@@ -25446,7 +25536,7 @@
       <c r="R111" s="58" t="inlineStr"/>
       <c r="S111" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T111" s="58" t="inlineStr">
@@ -25520,7 +25610,7 @@
       <c r="R112" s="58" t="inlineStr"/>
       <c r="S112" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T112" s="58" t="inlineStr">
@@ -25594,7 +25684,7 @@
       <c r="R113" s="58" t="inlineStr"/>
       <c r="S113" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T113" s="58" t="inlineStr">
@@ -25672,7 +25762,7 @@
       </c>
       <c r="S114" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T114" s="58" t="inlineStr">
@@ -25746,7 +25836,7 @@
       <c r="R115" s="58" t="inlineStr"/>
       <c r="S115" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T115" s="58" t="inlineStr">
@@ -25824,7 +25914,7 @@
       </c>
       <c r="S116" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T116" s="58" t="inlineStr">
@@ -25902,7 +25992,7 @@
       <c r="R117" s="58" t="inlineStr"/>
       <c r="S117" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T117" s="58" t="inlineStr">
@@ -25980,7 +26070,7 @@
       <c r="R118" s="58" t="inlineStr"/>
       <c r="S118" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T118" s="58" t="inlineStr">
@@ -26058,7 +26148,7 @@
       <c r="R119" s="58" t="inlineStr"/>
       <c r="S119" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T119" s="58" t="inlineStr">
@@ -26136,7 +26226,7 @@
       <c r="R120" s="58" t="inlineStr"/>
       <c r="S120" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T120" s="58" t="inlineStr">
@@ -26218,7 +26308,7 @@
       <c r="R121" s="58" t="inlineStr"/>
       <c r="S121" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T121" s="58" t="inlineStr">
@@ -26300,7 +26390,7 @@
       <c r="R122" s="58" t="inlineStr"/>
       <c r="S122" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T122" s="58" t="inlineStr">
@@ -26382,7 +26472,7 @@
       <c r="R123" s="58" t="inlineStr"/>
       <c r="S123" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T123" s="58" t="inlineStr">
@@ -26468,7 +26558,7 @@
       <c r="R124" s="58" t="inlineStr"/>
       <c r="S124" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T124" s="58" t="inlineStr">
@@ -26554,7 +26644,7 @@
       <c r="R125" s="58" t="inlineStr"/>
       <c r="S125" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T125" s="58" t="inlineStr">
@@ -26636,7 +26726,7 @@
       <c r="R126" s="58" t="inlineStr"/>
       <c r="S126" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T126" s="58" t="inlineStr">
@@ -26718,7 +26808,7 @@
       <c r="R127" s="58" t="inlineStr"/>
       <c r="S127" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T127" s="58" t="inlineStr">
@@ -26800,7 +26890,7 @@
       <c r="R128" s="58" t="inlineStr"/>
       <c r="S128" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T128" s="58" t="inlineStr">
@@ -26882,7 +26972,7 @@
       <c r="R129" s="58" t="inlineStr"/>
       <c r="S129" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T129" s="58" t="inlineStr">
@@ -26964,7 +27054,7 @@
       <c r="R130" s="58" t="inlineStr"/>
       <c r="S130" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T130" s="58" t="inlineStr">
@@ -27046,7 +27136,7 @@
       <c r="R131" s="58" t="inlineStr"/>
       <c r="S131" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T131" s="58" t="inlineStr">
@@ -27128,7 +27218,7 @@
       <c r="R132" s="58" t="inlineStr"/>
       <c r="S132" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T132" s="58" t="inlineStr">
@@ -27214,7 +27304,7 @@
       <c r="R133" s="58" t="inlineStr"/>
       <c r="S133" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T133" s="58" t="inlineStr">
@@ -27300,7 +27390,7 @@
       <c r="R134" s="58" t="inlineStr"/>
       <c r="S134" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T134" s="58" t="inlineStr">
@@ -27378,7 +27468,7 @@
       <c r="R135" s="58" t="inlineStr"/>
       <c r="S135" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T135" s="58" t="inlineStr">
@@ -27464,7 +27554,7 @@
       <c r="R136" s="58" t="inlineStr"/>
       <c r="S136" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T136" s="58" t="inlineStr">
@@ -27546,7 +27636,7 @@
       <c r="R137" s="58" t="inlineStr"/>
       <c r="S137" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T137" s="58" t="inlineStr">
@@ -27628,7 +27718,7 @@
       <c r="R138" s="58" t="inlineStr"/>
       <c r="S138" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T138" s="58" t="inlineStr">
@@ -27710,7 +27800,7 @@
       <c r="R139" s="58" t="inlineStr"/>
       <c r="S139" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T139" s="58" t="inlineStr">
@@ -27796,7 +27886,7 @@
       <c r="R140" s="58" t="inlineStr"/>
       <c r="S140" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T140" s="58" t="inlineStr">
@@ -27882,7 +27972,7 @@
       <c r="R141" s="58" t="inlineStr"/>
       <c r="S141" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T141" s="58" t="inlineStr">
@@ -27968,7 +28058,7 @@
       <c r="R142" s="58" t="inlineStr"/>
       <c r="S142" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T142" s="58" t="inlineStr">
@@ -28054,7 +28144,7 @@
       <c r="R143" s="58" t="inlineStr"/>
       <c r="S143" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T143" s="58" t="inlineStr">
@@ -28140,7 +28230,7 @@
       <c r="R144" s="58" t="inlineStr"/>
       <c r="S144" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T144" s="58" t="inlineStr">
@@ -28226,7 +28316,7 @@
       <c r="R145" s="58" t="inlineStr"/>
       <c r="S145" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T145" s="58" t="inlineStr">
@@ -28308,7 +28398,7 @@
       <c r="R146" s="58" t="inlineStr"/>
       <c r="S146" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T146" s="58" t="inlineStr">
@@ -28390,7 +28480,7 @@
       <c r="R147" s="58" t="inlineStr"/>
       <c r="S147" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T147" s="58" t="inlineStr">
@@ -28476,7 +28566,7 @@
       <c r="R148" s="58" t="inlineStr"/>
       <c r="S148" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T148" s="58" t="inlineStr">
@@ -28562,7 +28652,7 @@
       <c r="R149" s="58" t="inlineStr"/>
       <c r="S149" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T149" s="58" t="inlineStr">
@@ -28648,7 +28738,7 @@
       <c r="R150" s="58" t="inlineStr"/>
       <c r="S150" s="58" t="inlineStr">
         <is>
-          <t>v8.2</t>
+          <t>v8.3</t>
         </is>
       </c>
       <c r="T150" s="58" t="inlineStr">

</xml_diff>